<commit_message>
nexidoc: Purchasing audit — live click-through findings added (84 findings)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T49gnSNZq31rPRt1vHk4Rc
</commit_message>
<xml_diff>
--- a/nexidoc/Nexi_Purchasing_Audit_v21.49.xlsx
+++ b/nexidoc/Nexi_Purchasing_Audit_v21.49.xlsx
@@ -11,9 +11,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stores" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fix plan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Live click-through" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Findings'!$A$1:$J$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Findings'!$A$1:$J$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -589,7 +590,7 @@
         <v>5</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>0.07042253521126761</v>
+        <v>0.05952380952380952</v>
       </c>
     </row>
     <row r="7">
@@ -599,13 +600,13 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>0.2253521126760563</v>
+        <v>0.2380952380952381</v>
       </c>
     </row>
     <row r="8">
@@ -615,13 +616,13 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>0.4084507042253521</v>
+        <v>0.4166666666666667</v>
       </c>
     </row>
     <row r="9">
@@ -631,13 +632,13 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>0.2957746478873239</v>
+        <v>0.2857142857142857</v>
       </c>
     </row>
     <row r="10">
@@ -647,10 +648,10 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C10" s="11" t="n">
-        <v>71</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11">
@@ -792,13 +793,13 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="C20" s="6" t="n">
         <v>0</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
@@ -877,7 +878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J72"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4636,8 +4637,684 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" s="14" t="inlineStr">
+        <is>
+          <t>LV-01</t>
+        </is>
+      </c>
+      <c r="B73" s="14" t="inlineStr">
+        <is>
+          <t>Live click-through (Accounting screens)</t>
+        </is>
+      </c>
+      <c r="C73" s="14" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D73" s="16" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E73" s="14" t="inlineStr">
+        <is>
+          <t>~254870 (toolbar collapser)</t>
+        </is>
+      </c>
+      <c r="F73" s="14" t="inlineStr">
+        <is>
+          <t>The Workspace's 9-tab bar is swallowed by the global 'All tools' collapser 2–5 s after render: the 8 workflow tabs vanish into a dropdown under 'More'.</t>
+        </is>
+      </c>
+      <c r="G73" s="14" t="inlineStr">
+        <is>
+          <t>Open Purchasing, wait a few seconds, try to click RFQs or Invoices: the tabs are gone (live: click timed out, element hidden).</t>
+        </is>
+      </c>
+      <c r="H73" s="14" t="inlineStr">
+        <is>
+          <t>Exclude the purchasing nav from the collapser.</t>
+        </is>
+      </c>
+      <c r="I73" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J73" s="14" t="inlineStr">
+        <is>
+          <t>P1 consolidation</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="14" t="inlineStr">
+        <is>
+          <t>LV-02</t>
+        </is>
+      </c>
+      <c r="B74" s="14" t="inlineStr">
+        <is>
+          <t>Live click-through (Accounting screens)</t>
+        </is>
+      </c>
+      <c r="C74" s="14" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D74" s="16" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E74" s="14" t="inlineStr">
+        <is>
+          <t>sup360N modal; Cloud Fix banner</t>
+        </is>
+      </c>
+      <c r="F74" s="14" t="inlineStr">
+        <is>
+          <t>The Supplier 360° modal's ✕ sits under the fixed 'Cloud worker unreachable' banner and there is no Escape / backdrop close, so the whole screen is blocked once it opens.</t>
+        </is>
+      </c>
+      <c r="G74" s="14" t="inlineStr">
+        <is>
+          <t>Click any supplier name at Sourcing while a cloud banner shows: nothing on the screen can be clicked any more (live: run stopped here).</t>
+        </is>
+      </c>
+      <c r="H74" s="14" t="inlineStr">
+        <is>
+          <t>Backdrop click + Escape to close; modal above banners; same for the outreach and location modals.</t>
+        </is>
+      </c>
+      <c r="I74" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J74" s="14" t="inlineStr">
+        <is>
+          <t>P1 consolidation</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="14" t="inlineStr">
+        <is>
+          <t>LV-03</t>
+        </is>
+      </c>
+      <c r="B75" s="14" t="inlineStr">
+        <is>
+          <t>Live click-through (Accounting screens)</t>
+        </is>
+      </c>
+      <c r="C75" s="14" t="inlineStr">
+        <is>
+          <t>payment</t>
+        </is>
+      </c>
+      <c r="D75" s="16" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E75" s="14" t="inlineStr">
+        <is>
+          <t>~96770–96830; 97190</t>
+        </is>
+      </c>
+      <c r="F75" s="14" t="inlineStr">
+        <is>
+          <t>No payment stage exists: the chain advertised as PR → … → payment ends at invoice Approved.</t>
+        </is>
+      </c>
+      <c r="G75" s="14" t="inlineStr">
+        <is>
+          <t>Approve an invoice and look for Pay / Mark paid: nothing.</t>
+        </is>
+      </c>
+      <c r="H75" s="14" t="inlineStr">
+        <is>
+          <t>Paid state with date, reference, method; shown in cockpit and analytics.</t>
+        </is>
+      </c>
+      <c r="I75" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J75" s="14" t="inlineStr">
+        <is>
+          <t>P1 consolidation</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="14" t="inlineStr">
+        <is>
+          <t>LV-04</t>
+        </is>
+      </c>
+      <c r="B76" s="14" t="inlineStr">
+        <is>
+          <t>Live click-through (Accounting screens)</t>
+        </is>
+      </c>
+      <c r="C76" s="14" t="inlineStr">
+        <is>
+          <t>permissions</t>
+        </is>
+      </c>
+      <c r="D76" s="16" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E76" s="14" t="inlineStr">
+        <is>
+          <t>~96340; ~61313</t>
+        </is>
+      </c>
+      <c r="F76" s="14" t="inlineStr">
+        <is>
+          <t>Live: the admin created, submitted, AI-accepted and approved his own PR with no warning; the whole accounting role has managePayroll, so every accountant is a purchasing approver.</t>
+        </is>
+      </c>
+      <c r="G76" s="14" t="inlineStr">
+        <is>
+          <t>Jinky creates a PR and approves it herself.</t>
+        </is>
+      </c>
+      <c r="H76" s="14" t="inlineStr">
+        <is>
+          <t>Refuse approve/award/issue by the requester; dedicated approver permission.</t>
+        </is>
+      </c>
+      <c r="I76" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J76" s="14" t="inlineStr">
+        <is>
+          <t>P1 consolidation</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="14" t="inlineStr">
+        <is>
+          <t>LV-05</t>
+        </is>
+      </c>
+      <c r="B77" s="14" t="inlineStr">
+        <is>
+          <t>Live click-through (Accounting screens)</t>
+        </is>
+      </c>
+      <c r="C77" s="14" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D77" s="17" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E77" s="14" t="inlineStr">
+        <is>
+          <t>advance()</t>
+        </is>
+      </c>
+      <c r="F77" s="14" t="inlineStr">
+        <is>
+          <t>Approve, Reviewed, Verified and Run AI advance the stage silently (no toast); Submit, Accept and Override do.</t>
+        </is>
+      </c>
+      <c r="G77" s="14" t="inlineStr">
+        <is>
+          <t>Click Approve at Department Approval: nothing visibly happens except a chip change.</t>
+        </is>
+      </c>
+      <c r="H77" s="14" t="inlineStr">
+        <is>
+          <t>Toast on every stage change.</t>
+        </is>
+      </c>
+      <c r="I77" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J77" s="14" t="inlineStr">
+        <is>
+          <t>P1 consolidation</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="14" t="inlineStr">
+        <is>
+          <t>LV-06</t>
+        </is>
+      </c>
+      <c r="B78" s="14" t="inlineStr">
+        <is>
+          <t>Live click-through (Accounting screens)</t>
+        </is>
+      </c>
+      <c r="C78" s="14" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D78" s="17" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E78" s="14" t="inlineStr">
+        <is>
+          <t>rInvoices()</t>
+        </is>
+      </c>
+      <c r="F78" s="14" t="inlineStr">
+        <is>
+          <t>Invoices tab shows an empty PO select on a fresh install; the only guard is 'PO, invoice number and amount are required.'</t>
+        </is>
+      </c>
+      <c r="G78" s="14" t="inlineStr">
+        <is>
+          <t>Fresh install → Invoices → Log &amp; match → cryptic alert.</t>
+        </is>
+      </c>
+      <c r="H78" s="14" t="inlineStr">
+        <is>
+          <t>Show 'Issue a purchase order first' and disable the button.</t>
+        </is>
+      </c>
+      <c r="I78" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J78" s="14" t="inlineStr">
+        <is>
+          <t>P1 consolidation</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="14" t="inlineStr">
+        <is>
+          <t>LV-07</t>
+        </is>
+      </c>
+      <c r="B79" s="14" t="inlineStr">
+        <is>
+          <t>Live click-through (Accounting screens)</t>
+        </is>
+      </c>
+      <c r="C79" s="14" t="inlineStr">
+        <is>
+          <t>sourcing</t>
+        </is>
+      </c>
+      <c r="D79" s="17" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E79" s="14" t="inlineStr">
+        <is>
+          <t>rSourcing()</t>
+        </is>
+      </c>
+      <c r="F79" s="14" t="inlineStr">
+        <is>
+          <t>With an empty vendor master, Sourcing shows 'Nexi found 0 candidates' and offers no way to add a supplier; the only exit is 'Pick at least one supplier.'</t>
+        </is>
+      </c>
+      <c r="G79" s="14" t="inlineStr">
+        <is>
+          <t>First procurement on a device with no vendors is a dead end.</t>
+        </is>
+      </c>
+      <c r="H79" s="14" t="inlineStr">
+        <is>
+          <t>'Add supplier' inline and a link to the supplier master.</t>
+        </is>
+      </c>
+      <c r="I79" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J79" s="14" t="inlineStr">
+        <is>
+          <t>P1 consolidation</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="14" t="inlineStr">
+        <is>
+          <t>LV-08</t>
+        </is>
+      </c>
+      <c r="B80" s="14" t="inlineStr">
+        <is>
+          <t>Live click-through (Accounting screens)</t>
+        </is>
+      </c>
+      <c r="C80" s="14" t="inlineStr">
+        <is>
+          <t>cockpit</t>
+        </is>
+      </c>
+      <c r="D80" s="17" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E80" s="14" t="inlineStr">
+        <is>
+          <t>277798 / 277826 / 277850</t>
+        </is>
+      </c>
+      <c r="F80" s="14" t="inlineStr">
+        <is>
+          <t>All three Accounting cockpit boxes (Purchase requests, POs &amp; receiving, Supplier invoices) open the same Mission Control tab.</t>
+        </is>
+      </c>
+      <c r="G80" s="14" t="inlineStr">
+        <is>
+          <t>Click 'Supplier invoices' on the cockpit → lands on Mission Control, numbers do not match.</t>
+        </is>
+      </c>
+      <c r="H80" s="14" t="inlineStr">
+        <is>
+          <t>Open the matching tab (pos / invs).</t>
+        </is>
+      </c>
+      <c r="I80" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J80" s="14" t="inlineStr">
+        <is>
+          <t>P1 consolidation</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="14" t="inlineStr">
+        <is>
+          <t>LV-09</t>
+        </is>
+      </c>
+      <c r="B81" s="14" t="inlineStr">
+        <is>
+          <t>Live click-through (Accounting screens)</t>
+        </is>
+      </c>
+      <c r="C81" s="14" t="inlineStr">
+        <is>
+          <t>AI gate</t>
+        </is>
+      </c>
+      <c r="D81" s="17" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E81" s="14" t="inlineStr">
+        <is>
+          <t>analyzePR() ~96600</t>
+        </is>
+      </c>
+      <c r="F81" s="14" t="inlineStr">
+        <is>
+          <t>'AI Validation' is a rules check (stock hint, history average, duplicate PR); with no data it always says 'Purchase required. 88%'.</t>
+        </is>
+      </c>
+      <c r="G81" s="14" t="inlineStr">
+        <is>
+          <t>Every first PR shows a confident percentage that means nothing.</t>
+        </is>
+      </c>
+      <c r="H81" s="14" t="inlineStr">
+        <is>
+          <t>Label it 'Rules check' or route through the Nexi brain worker.</t>
+        </is>
+      </c>
+      <c r="I81" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J81" s="14" t="inlineStr">
+        <is>
+          <t>P1 consolidation</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="14" t="inlineStr">
+        <is>
+          <t>LV-10</t>
+        </is>
+      </c>
+      <c r="B82" s="14" t="inlineStr">
+        <is>
+          <t>Live click-through (Accounting screens)</t>
+        </is>
+      </c>
+      <c r="C82" s="14" t="inlineStr">
+        <is>
+          <t>dates</t>
+        </is>
+      </c>
+      <c r="D82" s="18" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="E82" s="14" t="inlineStr">
+        <is>
+          <t>~96335</t>
+        </is>
+      </c>
+      <c r="F82" s="14" t="inlineStr">
+        <is>
+          <t>Dates use UTC toISOString, not hnxLocalToday(); after 16:00 Manila every date is one day early.</t>
+        </is>
+      </c>
+      <c r="G82" s="14" t="inlineStr">
+        <is>
+          <t>GRN recorded at 19:00 PHT gets yesterday's date.</t>
+        </is>
+      </c>
+      <c r="H82" s="14" t="inlineStr">
+        <is>
+          <t>Use hnxLocalToday().</t>
+        </is>
+      </c>
+      <c r="I82" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J82" s="14" t="inlineStr">
+        <is>
+          <t>P1 consolidation</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="14" t="inlineStr">
+        <is>
+          <t>LV-11</t>
+        </is>
+      </c>
+      <c r="B83" s="14" t="inlineStr">
+        <is>
+          <t>Live click-through (Accounting screens)</t>
+        </is>
+      </c>
+      <c r="C83" s="14" t="inlineStr">
+        <is>
+          <t>3-way match</t>
+        </is>
+      </c>
+      <c r="D83" s="18" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="E83" s="14" t="inlineStr">
+        <is>
+          <t>award() ~97120; matchInvoice() ~96770</t>
+        </is>
+      </c>
+      <c r="F83" s="14" t="inlineStr">
+        <is>
+          <t>Scaled, rounded line prices no longer sum to the PO total; rounding alone can push a correct invoice into 'Waiting GRN'.</t>
+        </is>
+      </c>
+      <c r="G83" s="14" t="inlineStr">
+        <is>
+          <t>Estimate ₱2,500, quote ₱2,599.99, 3 lines → mismatch.</t>
+        </is>
+      </c>
+      <c r="H83" s="14" t="inlineStr">
+        <is>
+          <t>Match by quantity, or put the rounding remainder on the last line.</t>
+        </is>
+      </c>
+      <c r="I83" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J83" s="14" t="inlineStr">
+        <is>
+          <t>P1 consolidation</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="14" t="inlineStr">
+        <is>
+          <t>LV-12</t>
+        </is>
+      </c>
+      <c r="B84" s="14" t="inlineStr">
+        <is>
+          <t>Live click-through (Accounting screens)</t>
+        </is>
+      </c>
+      <c r="C84" s="14" t="inlineStr">
+        <is>
+          <t>duplication</t>
+        </is>
+      </c>
+      <c r="D84" s="17" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E84" s="14" t="inlineStr">
+        <is>
+          <t>_purchAward ~95690; sendRFQ ~96885</t>
+        </is>
+      </c>
+      <c r="F84" s="14" t="inlineStr">
+        <is>
+          <t>Quick Tools has its own comparisons / outreach / history with its own 'award'; an awarded comparison never creates a PR or PO; Workspace RFQ sends land in the outreach log with qty 0.</t>
+        </is>
+      </c>
+      <c r="G84" s="14" t="inlineStr">
+        <is>
+          <t>Award a comparison in Quick Tools, then look at Purchase Orders: nothing.</t>
+        </is>
+      </c>
+      <c r="H84" s="14" t="inlineStr">
+        <is>
+          <t>'Convert to request' on an awarded comparison; one outreach record shape.</t>
+        </is>
+      </c>
+      <c r="I84" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J84" s="14" t="inlineStr">
+        <is>
+          <t>P1 consolidation</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="14" t="inlineStr">
+        <is>
+          <t>LV-13</t>
+        </is>
+      </c>
+      <c r="B85" s="14" t="inlineStr">
+        <is>
+          <t>Live click-through (Accounting screens)</t>
+        </is>
+      </c>
+      <c r="C85" s="14" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D85" s="18" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="E85" s="14" t="inlineStr">
+        <is>
+          <t>Cloud Fix banner</t>
+        </is>
+      </c>
+      <c r="F85" s="14" t="inlineStr">
+        <is>
+          <t>The red 'Cloud worker unreachable' banner stays pinned over every screen and overlaps modals.</t>
+        </is>
+      </c>
+      <c r="G85" s="14" t="inlineStr">
+        <is>
+          <t>Any offline minute makes modals unclosable (LV-02).</t>
+        </is>
+      </c>
+      <c r="H85" s="14" t="inlineStr">
+        <is>
+          <t>Collapse to a status chip after first dismissal; keep it below modals.</t>
+        </is>
+      </c>
+      <c r="I85" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J85" s="14" t="inlineStr">
+        <is>
+          <t>P1 consolidation</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J72"/>
+  <autoFilter ref="A1:J85"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5430,4 +6107,288 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Has handler</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>What happened</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Workspace</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>🎯 Mission Control / 📝 Requests / 📨 RFQs / 📄 POs / 📦 Receiving / 🧾 Invoices / 🏭 Scorecard / 📈 Analytics / ↩ Quick tools</t>
+        </is>
+      </c>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>All render (empty states). RFQs and Invoices tabs had already been hidden by the toolbar collapser and had to be clicked via script (LV-01).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>Workspace</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>➕ New Purchase Request → 💾 Save Draft</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>Sequential alerts for title, dept, need-by, justification ≥30 chars, ≥1 line; then 'Created PR-2026-000001' with the 13-chip pipeline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Workspace</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>🚀 Submit → 🤖 Run AI analysis → ✅ Accept / ❌ Reject to Draft / ✋ Override</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>All work; AI panel 'SOS on-hand 0 · past buys 0 → Purchase required. 88%' (LV-09); reject returns to Draft with log; override advances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>Workspace</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>✅ Approve (dept) → ✅ Reviewed → ✅ Verified</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>Advance silently, no toast (LV-05); the same admin approved his own PR (LV-04).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Workspace</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Supplier Sourcing: candidates, select-all, 📨 Create RFQ, Supplier 360°</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>0 candidates with an empty vendor master (LV-07); after seeding 3 vendors the table lists them; 360° opens but cannot be closed under the cloud banner (LV-02) — run blocked here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>Workspace</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>RFQ send / quotes / evaluation / award / Issue PO / amendment / GRN / complete / invoice log &amp; match / approve / force approve</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>NOT REACHED live (blocked by LV-02); handlers exist and were code-reviewed (PW-xx findings).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Workspace</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>🧾 Invoices → 💾 Log &amp; match (fresh install)</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Empty PO select; alert 'PO, invoice number and amount are required.' (LV-06).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Quick Tools</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>📥 Sync purchase history from SOS</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Disabled offline with tooltip 'Connect SOS in Admin → SOS Inventory Sync first' — honest (needs network).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Quick Tools</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Comparisons / History / Suppliers Ledger / RFQ Log / outreach modal / location &amp; radius / export CSV</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>NOT REACHED live (harness stopped); all have handlers; findings QT-xx from code review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Accounting cockpit</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Purchase requests / POs &amp; receiving / Supplier invoices boxes</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>All three go to the same Mission Control tab (LV-08).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Jinky (accounting role)</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Create and approve own PR</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>NOT REACHED live; by code she can (LV-04 / PW-02).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>